<commit_message>
crud basic in express but error :(
</commit_message>
<xml_diff>
--- a/documents/felicette_server.xlsx
+++ b/documents/felicette_server.xlsx
@@ -1,22 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\workspace\felicette_server\documents\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\work\felicette\felicette_server\documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EB3D4A12-8E3F-43FF-B7D9-9B1C944027E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="3"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15990" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="API" sheetId="1" r:id="rId1"/>
     <sheet name="browser extension" sheetId="5" r:id="rId2"/>
     <sheet name="screen" sheetId="2" r:id="rId3"/>
     <sheet name="DB" sheetId="3" r:id="rId4"/>
-    <sheet name="settup" sheetId="4" r:id="rId5"/>
+    <sheet name="settup and document" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="141">
   <si>
     <t>API</t>
   </si>
@@ -766,11 +767,17 @@
   <si>
     <t>phone</t>
   </si>
+  <si>
+    <t>https://github.com/daniel7byte/base-nodejs-project-gcp/blob/main/src/services/country.js</t>
+  </si>
+  <si>
+    <t>xem chi tiet mo hinh mvc</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -940,7 +947,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -984,7 +991,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -2703,137 +2709,137 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:AA110"/>
   <sheetFormatPr defaultColWidth="4.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="1" spans="1:27" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="C1" s="23"/>
-      <c r="D1" s="23"/>
-      <c r="E1" s="23"/>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23" t="s">
+      <c r="B1" s="22"/>
+      <c r="C1" s="22"/>
+      <c r="D1" s="22"/>
+      <c r="E1" s="22"/>
+      <c r="F1" s="22"/>
+      <c r="G1" s="22"/>
+      <c r="H1" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23" t="s">
+      <c r="I1" s="22"/>
+      <c r="J1" s="22"/>
+      <c r="K1" s="22"/>
+      <c r="L1" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="23"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="23"/>
-      <c r="U1" s="23"/>
-      <c r="V1" s="23"/>
-      <c r="W1" s="23"/>
-      <c r="X1" s="23"/>
-      <c r="Y1" s="23"/>
-      <c r="Z1" s="23"/>
-      <c r="AA1" s="23"/>
+      <c r="M1" s="22"/>
+      <c r="N1" s="22"/>
+      <c r="O1" s="22"/>
+      <c r="P1" s="22"/>
+      <c r="Q1" s="22"/>
+      <c r="R1" s="22"/>
+      <c r="S1" s="22"/>
+      <c r="T1" s="22"/>
+      <c r="U1" s="22"/>
+      <c r="V1" s="22"/>
+      <c r="W1" s="22"/>
+      <c r="X1" s="22"/>
+      <c r="Y1" s="22"/>
+      <c r="Z1" s="22"/>
+      <c r="AA1" s="22"/>
     </row>
     <row r="2" spans="1:27" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="24" t="s">
+      <c r="A2" s="23" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="24"/>
-      <c r="C2" s="24"/>
-      <c r="D2" s="24"/>
-      <c r="E2" s="24"/>
-      <c r="F2" s="24"/>
-      <c r="G2" s="24"/>
-      <c r="H2" s="24" t="s">
+      <c r="B2" s="23"/>
+      <c r="C2" s="23"/>
+      <c r="D2" s="23"/>
+      <c r="E2" s="23"/>
+      <c r="F2" s="23"/>
+      <c r="G2" s="23"/>
+      <c r="H2" s="23" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="24"/>
-      <c r="J2" s="24"/>
-      <c r="K2" s="24"/>
-      <c r="L2" s="24" t="s">
+      <c r="I2" s="23"/>
+      <c r="J2" s="23"/>
+      <c r="K2" s="23"/>
+      <c r="L2" s="23" t="s">
         <v>3</v>
       </c>
-      <c r="M2" s="24"/>
-      <c r="N2" s="24"/>
-      <c r="O2" s="24"/>
-      <c r="P2" s="24"/>
-      <c r="Q2" s="24"/>
-      <c r="R2" s="24"/>
-      <c r="S2" s="24"/>
-      <c r="T2" s="24"/>
-      <c r="U2" s="24"/>
-      <c r="V2" s="24"/>
-      <c r="W2" s="24"/>
-      <c r="X2" s="24"/>
-      <c r="Y2" s="24"/>
-      <c r="Z2" s="24"/>
-      <c r="AA2" s="24"/>
+      <c r="M2" s="23"/>
+      <c r="N2" s="23"/>
+      <c r="O2" s="23"/>
+      <c r="P2" s="23"/>
+      <c r="Q2" s="23"/>
+      <c r="R2" s="23"/>
+      <c r="S2" s="23"/>
+      <c r="T2" s="23"/>
+      <c r="U2" s="23"/>
+      <c r="V2" s="23"/>
+      <c r="W2" s="23"/>
+      <c r="X2" s="23"/>
+      <c r="Y2" s="23"/>
+      <c r="Z2" s="23"/>
+      <c r="AA2" s="23"/>
     </row>
     <row r="4" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="21" t="s">
         <v>20</v>
       </c>
-      <c r="C4" s="22"/>
-      <c r="D4" s="22"/>
-      <c r="E4" s="22"/>
-      <c r="F4" s="22"/>
-      <c r="G4" s="22"/>
-      <c r="H4" s="22"/>
-      <c r="I4" s="22"/>
-      <c r="J4" s="22"/>
-      <c r="K4" s="22"/>
-      <c r="L4" s="22"/>
-      <c r="M4" s="22"/>
-      <c r="N4" s="22"/>
-      <c r="O4" s="22"/>
-      <c r="P4" s="22"/>
-      <c r="Q4" s="22"/>
-      <c r="R4" s="22"/>
-      <c r="S4" s="22"/>
-      <c r="T4" s="22"/>
-      <c r="U4" s="22"/>
-      <c r="V4" s="22"/>
-      <c r="W4" s="22"/>
-      <c r="X4" s="22"/>
-      <c r="Y4" s="22"/>
-      <c r="Z4" s="22"/>
-      <c r="AA4" s="22"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
+      <c r="Y4" s="21"/>
+      <c r="Z4" s="21"/>
+      <c r="AA4" s="21"/>
     </row>
     <row r="5" spans="1:27" x14ac:dyDescent="0.25">
-      <c r="B5" s="22"/>
-      <c r="C5" s="22"/>
-      <c r="D5" s="22"/>
-      <c r="E5" s="22"/>
-      <c r="F5" s="22"/>
-      <c r="G5" s="22"/>
-      <c r="H5" s="22"/>
-      <c r="I5" s="22"/>
-      <c r="J5" s="22"/>
-      <c r="K5" s="22"/>
-      <c r="L5" s="22"/>
-      <c r="M5" s="22"/>
-      <c r="N5" s="22"/>
-      <c r="O5" s="22"/>
-      <c r="P5" s="22"/>
-      <c r="Q5" s="22"/>
-      <c r="R5" s="22"/>
-      <c r="S5" s="22"/>
-      <c r="T5" s="22"/>
-      <c r="U5" s="22"/>
-      <c r="V5" s="22"/>
-      <c r="W5" s="22"/>
-      <c r="X5" s="22"/>
-      <c r="Y5" s="22"/>
-      <c r="Z5" s="22"/>
-      <c r="AA5" s="22"/>
+      <c r="B5" s="21"/>
+      <c r="C5" s="21"/>
+      <c r="D5" s="21"/>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21"/>
+      <c r="G5" s="21"/>
+      <c r="H5" s="21"/>
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+      <c r="L5" s="21"/>
+      <c r="M5" s="21"/>
+      <c r="N5" s="21"/>
+      <c r="O5" s="21"/>
+      <c r="P5" s="21"/>
+      <c r="Q5" s="21"/>
+      <c r="R5" s="21"/>
+      <c r="S5" s="21"/>
+      <c r="T5" s="21"/>
+      <c r="U5" s="21"/>
+      <c r="V5" s="21"/>
+      <c r="W5" s="21"/>
+      <c r="X5" s="21"/>
+      <c r="Y5" s="21"/>
+      <c r="Z5" s="21"/>
+      <c r="AA5" s="21"/>
     </row>
     <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="B6" s="11" t="s">
@@ -3125,67 +3131,67 @@
       <c r="C52" s="12"/>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D53" s="21" t="s">
+      <c r="D53" s="20" t="s">
         <v>115</v>
       </c>
     </row>
     <row r="55" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D55" s="20" t="s">
+      <c r="D55" s="19" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="56" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D56" s="20" t="s">
+      <c r="D56" s="19" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="57" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D57" s="20" t="s">
+      <c r="D57" s="19" t="s">
         <v>113</v>
       </c>
     </row>
     <row r="58" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="D58" s="20" t="s">
+      <c r="D58" s="19" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="103" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="B103" s="19" t="s">
+      <c r="B103" s="12" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="104" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C104" s="21" t="s">
+      <c r="C104" s="20" t="s">
         <v>114</v>
       </c>
     </row>
     <row r="105" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C105" s="20" t="s">
+      <c r="C105" s="19" t="s">
         <v>106</v>
       </c>
     </row>
     <row r="106" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C106" s="20" t="s">
+      <c r="C106" s="19" t="s">
         <v>107</v>
       </c>
     </row>
     <row r="107" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C107" s="20" t="s">
+      <c r="C107" s="19" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="108" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C108" s="20" t="s">
+      <c r="C108" s="19" t="s">
         <v>109</v>
       </c>
     </row>
     <row r="109" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C109" s="20" t="s">
+      <c r="C109" s="19" t="s">
         <v>110</v>
       </c>
     </row>
     <row r="110" spans="2:3" x14ac:dyDescent="0.25">
-      <c r="C110" s="20" t="s">
+      <c r="C110" s="19" t="s">
         <v>111</v>
       </c>
     </row>
@@ -3207,7 +3213,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A3:B3"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3226,7 +3232,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="B30:R89"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -3399,7 +3405,7 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B2:AA69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -3864,8 +3870,8 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B2:B5"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
+  <dimension ref="B2:B10"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="2" spans="2:2" x14ac:dyDescent="0.25">
@@ -3888,6 +3894,16 @@
         <v>35</v>
       </c>
     </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B9" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="B10" t="s">
+        <v>139</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>